<commit_message>
Log rejected candidates in the stance-update audit trail
Ran the verify-and-apply pass over every finding surfaced this session,
not just the two already applied. Everything else (settlement tax law,
land-registration order, communications law, deserter-arrest bill,
Eisenkot campaign launch, Goldknopf/Gafni vs. AG, Bennett's economic
plan, Gantz's inquiry-commission remark, an unverified Liberman
allegation, and a batch of coalition/list-mechanics noise) failed
verification — mostly for falling outside the 7-day window - and is
now logged with its rejection reason instead of silently dropped.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZWGbfG1hwb137JuoH5rTt
</commit_message>
<xml_diff>
--- a/reports/party-stance-updates.xlsx
+++ b/reports/party-stance-updates.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
         <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE8E6"/>
+        <bgColor rgb="00FCE8E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,12 +82,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -449,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -545,7 +554,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>אומת — קיים מקור אמין ותאריך בתוך 7 הימים; הערך לא השתנה אך נוסף מקור</t>
+          <t>אומת ויושם</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -593,7 +602,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>אומת — כותרת ותוכן תואמים בשלושה מקורות חיפוש נפרדים; תאריך בתוך 7 הימים</t>
+          <t>אומת ויושם</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -609,6 +618,526 @@
       <c r="J3" s="2" t="inlineStr">
         <is>
           <t>כן — party_stances.ts עודכן (stanceValue 1→2, נוסף sourceUrl+sourceNote)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>likud / religious-zionism</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>sec-1</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>יש להרחיב את ההתיישבות היהודית ביהודה ושומרון.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>נפסל — מחוץ לחלון 7 הימים</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.inn.co.il/news/698314</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>חוק הטבות מס ליישובי קו עימות ביו"ש עבר קריאה שנייה/שלישית ב-4.6.2026, ופורסם 8.6.2026 — כחודשיים לפני הסריקה, לא אירוע של השבוע האחרון.</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>לא — נפסל באימות</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>religious-zionism / likud</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>sec-1 / sec-6</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>יש להרחיב את ההתיישבות... / יש לשמור על אחיזה ביטחונית קבועה ביו"ש.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>נפסל — מחוץ לחלון 7 הימים</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.makorrishon.co.il/news/settlement/article/307517</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>החלטת הממשלה על חידוש הסדר המקרקעין ביו"ש (סמוטריץ'/כ"ץ) התקבלה בפברואר 2026, כחצי שנה לפני הסריקה.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>לא — נפסל באימות</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>likud</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>gov-5</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>יש להגביל בעלות צולבת על תקשורת ולחזק את השידור הציבורי.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>נפסל — מחוץ לחלון 7 הימים</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ynet.co.il/news/article/rjbbarlege</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>חוק התקשורת של קרעי אושר סופית בכנסת (53-48) כשלושה שבועות לפני הסריקה (אמצע יולי 2026), לא בתוך 7 הימים.</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>לא — נפסל באימות</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>shas / yahadut-hatorah</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>rel-5</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>יש לשמר את פטור הגיוס לתלמידי ישיבות.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>נפסל — מחוץ לחלון 7 הימים</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ynet.co.il/news/article/rjp00xpz4mg</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>מכתב הרמטכ"ל נגד חוק הקפאת מעצרי העריקים ואישור ועדת החוץ והביטחון — תחילת יולי 2026, לא בתוך 7 הימים.</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>לא — נפסל באימות</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>yashar</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>rel-5</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>יש לשמר את פטור הגיוס לתלמידי ישיבות.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>נפסל — מחוץ לחלון 7 הימים</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mako.co.il/news-israel-elections/2026/Article-ba49072ad691f91027.htm</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>השקת קמפיין הבחירות של איזנקוט וחוק "שירות לכול" — מאי-יוני 2026, לא אירוע של השבוע האחרון.</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>לא — נפסל באימות</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>shas / yahadut-hatorah</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>jud-8</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>יש לשמר את מעמד היועץ המשפטי לממשלה כגורם מייעץ בלתי תלוי.</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>נפסל — מחוץ לחלון 7 הימים</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ynet.co.il/news/article/h1yh11ikr11e</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>עימות גולדקנופף/גפני מול היועמ"שית בנושא זיכוי מס לתורמי ישיבות — 29.4.2026, לא בתוך 7 הימים.</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>לא — נפסל באימות</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>beyachad</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>eco-12</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>יש לפתוח את השוק ליבוא חופשי כדי להוזיל את יוקר המחיה.</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>נפסל — מחוץ לחלון 7 הימים</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mako.co.il/news-money/2026_q2/Article-54fd6f938c81f91026.htm</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>תוכנית הכלכלית של בנט (פירוק מונופול תנובה, יבוא פירות/ירקות) — יוני 2026, לא אירוע של השבוע האחרון.</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>לא — נפסל באימות</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>kachol-lavan</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>gov-1</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>יש להקים ועדת חקירה ממלכתית לאירועי 7 באוקטובר.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>נפסל — לא אותר תאריך מאמת בתוך 7 הימים</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.maariv.co.il/breaking-news/article-1252867</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>הצהרת גנץ נגד 'הצעת פשרה' על הרכב ועדת חקירה — התאריך לא אומת כחל בשבוע 9-16.8.2026; חוזרת על עמדה קיימת ומתועדת, לא ממצא חדש.</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>לא — נפסל באימות</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>yisrael-beiteinu</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>sec-9 (חלקי)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>יש להעביר את השליטה האזרחית ברצועת עזה לגורם בינלאומי/ערבי.</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>נפסל — טענה לא מאומתת / אינה הצהרת מדיניות עצמאית</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>https://news.walla.co.il/item/3860235</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>טענת ליברמן על "עסקת 400 מיליון דולר עם חמאס" היא האשמה חמורה שלא אומתה במקור עצמאי, ולא הצהרת עמדה עקבית — לא נכלל.</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>לא — נפסל באימות</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>likud / yashar / raam / yisrael-beiteinu</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>אין שאלת סקר תואמת</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>נפסל — רעש קואליציוני/פנים-מפלגתי</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>השתלטות נתניהו על רשימת הליכוד בפריימריז; תוכנית ממשלת המיעוט של איזנקוט; סירוב ליברמן לשבת עם ש"ס/יהדות התורה/רע"ם; היפרדות רע"ם מהתנועה האסלאמית; ויתור גולן על השריונים ברשימה — כולם דינמיקת גוש/רשימה/קואליציה או ענייני פנים-מפלגתיים, מחוץ להיקף המתועד בראש party_stances.ts.</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>לא — מחוץ להיקף מלכתחילה</t>
         </is>
       </c>
     </row>

</xml_diff>